<commit_message>
commit with working BSCR query
</commit_message>
<xml_diff>
--- a/reporting/lloyds/workbooks/UKEU - Supplementary Info - RDL - Jan26 - Workings - California WF.xlsx
+++ b/reporting/lloyds/workbooks/UKEU - Supplementary Info - RDL - Jan26 - Workings - California WF.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath url="W:\Data\Cat Modelling\Group Reporting\Reports\2026\2026-01 - RDS\Supplementary Information\2. Data Received\Nat Cat\UKEU\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Data\Cat Modelling\Group Reporting\Reports\2026\2026-01 - RDS\Supplementary Information\2. Data Received\Nat Cat\UKEU\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF1C5BD3-70BB-4F31-ACC1-ABE2C2742450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19814" windowHeight="15990" tabRatio="773" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19814" windowHeight="15990" tabRatio="773" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="06 California Wildfire Aggs" sheetId="11" r:id="rId1"/>
     <sheet name="Core data" sheetId="2" r:id="rId2"/>
-    <sheet name="AUDIT_SUMMARY" sheetId="12" r:id="rId9"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId3"/>
@@ -31,7 +30,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
@@ -7696,138 +7695,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <cols>
-    <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="110" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>AUDIT SUMMARY</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>UKEU - Supplementary Info - RDL - Jan26 - Workings - California WF.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Purpose</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Produce California wildfire exposure by county.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>January 2026 working file with a legacy 01/01/2025 report label; cached values are preserved.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Sources</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Weather exposure/proxy decision or the structurally matching FA_California_Aggs.sql extract.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Process</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Populate Core data A:M. Helper column N extracts county text and the county report sums net USD exposure from column M.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Outputs</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>California county report, followed by reviewed manual template handoff.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Required control</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>The source email says wildfire was not monitored separately. Obtain approval for the proxy/PML and correct as-of date before use.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>January baseline SHA-256</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>36267a772d2a4252286d891556541296364a4bab15f028cee4dd6fd84fd9f0e8</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Run record</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Record server, database, codes, row count, totals, FX, operator, reviewer and date.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Start at docs/index.md. This sheet is a guide, not regulatory approval.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:B10"/>
-</worksheet>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{b0e772fd-230e-46a1-9b91-16e31ba7e038}" enabled="1" method="Privileged" siteId="{dfbcc178-bccf-4595-8f8e-3a3175df90b7}" contentBits="0" removed="0"/>

</xml_diff>